<commit_message>
Rename and organize all partner logo images to matching store slugs, and update Excel spreadsheet data
</commit_message>
<xml_diff>
--- a/sodanca-france-airtable-import.xlsx
+++ b/sodanca-france-airtable-import.xlsx
@@ -1027,7 +1027,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>237053185_4195401820543960_5789685567708466628_n-1.jpg</t>
+          <t>flashdance.jpg</t>
         </is>
       </c>
     </row>
@@ -1084,7 +1084,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>265653179_1317117552049587_6123476178514824761_n.png</t>
+          <t>la-danse.png</t>
         </is>
       </c>
     </row>
@@ -1104,7 +1104,6 @@
           <t>4, Rue Durand</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>33 467 920 370</t>
@@ -1115,12 +1114,9 @@
           <t>bolero.m@free.fr</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>boneco-so-danca-400x400-2.jpg</t>
+          <t>bolero.jpg</t>
         </is>
       </c>
     </row>
@@ -1177,7 +1173,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>301677157_491498676312784_1201436729283311743_n.jpg</t>
+          <t>esprit-studio.jpg</t>
         </is>
       </c>
     </row>
@@ -1202,7 +1198,6 @@
           <t>130, Chemin Sous St Etienne, Rond Point Rte de Bagnols</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>04 66 40 20 56</t>
@@ -1213,7 +1208,6 @@
           <t>flashdanse30@hotmail.com</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>https://www.facebook.com/FlashDanse30/</t>
@@ -1226,7 +1220,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>241342565_363970131832603_2608823694376204499_n.png</t>
+          <t>flash-danse.png</t>
         </is>
       </c>
     </row>
@@ -1266,16 +1260,14 @@
           <t>jpierrerey@yahoo.fr</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>https://www.facebook.com/ReyDanceShop/</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
-          <t>boneco-so-danca-400x400-2.jpg</t>
+          <t>rey-dance.jpg</t>
         </is>
       </c>
     </row>
@@ -1315,16 +1307,14 @@
           <t>passion.danse.contact@gmail.com</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
           <t>https://www.facebook.com/boutiquepassiondanse/</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>299685090_505750971552579_1833210039737964385_n.jpg</t>
+          <t>passion-danse.jpg</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1339,6 @@
           <t>250, Faubourg Saint Honoré</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>+33 1 45 62 37 95</t>
@@ -1377,7 +1366,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>292172165_464909825638627_7789637463979927889_n.png</t>
+          <t>stanlowa-3.png</t>
         </is>
       </c>
     </row>
@@ -1402,7 +1391,6 @@
           <t>6 Allee Vivaldi - Le Ny Christelle</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>06 20 49 46 84</t>
@@ -1413,16 +1401,14 @@
           <t>kidanse@live.fr</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
           <t>https://www.facebook.com/kidanse?ref=hl</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>305966223_520741190051489_277726456098938900_n.jpg</t>
+          <t>ki-danse.jpg</t>
         </is>
       </c>
     </row>
@@ -1479,7 +1465,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>448615550_2386439431561551_3591327418131567780_n.jpg</t>
+          <t>danse-boutic-avenue.jpg</t>
         </is>
       </c>
     </row>
@@ -1536,7 +1522,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>programar-europa-5.jpg</t>
+          <t>glace-danse.jpg</t>
         </is>
       </c>
     </row>
@@ -1576,7 +1562,6 @@
           <t>info@chorelys.com</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
           <t>https://www.facebook.com/chorelys/</t>
@@ -1589,7 +1574,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>programar-europa.jpg</t>
+          <t>chorelys.jpg</t>
         </is>
       </c>
     </row>
@@ -1639,10 +1624,9 @@
           <t>https://www.facebook.com/bodylangage/</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
-          <t>10174796_748751015175858_3332565469240181698_n.jpg</t>
+          <t>body-langage.jpg</t>
         </is>
       </c>
     </row>
@@ -1682,8 +1666,6 @@
           <t>cendryllon@orange.fr</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr">
         <is>
           <t>https://cendryllon.fr/</t>
@@ -1691,7 +1673,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>20240510_113058-768x354-1.jpg</t>
+          <t>cendryllon.jpg</t>
         </is>
       </c>
     </row>
@@ -1716,7 +1698,6 @@
           <t>10, Avenue Georges Clémenceau</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>33 147 081 680</t>
@@ -1727,7 +1708,6 @@
           <t>contact@lentrechats.fr</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>https://www.facebook.com/LEntrechats/</t>
@@ -1740,7 +1720,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>161812589_185023226758872_5130441343176373562_n.jpg</t>
+          <t>lentre-chats.jpg</t>
         </is>
       </c>
     </row>
@@ -1797,7 +1777,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>253549859_1988181661359089_8994290927255086920_n.png</t>
+          <t>danses-et-plage.png</t>
         </is>
       </c>
     </row>
@@ -1817,7 +1797,6 @@
           <t>4, Allée du Cadran</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>33 559 630 073</t>
@@ -1828,12 +1807,9 @@
           <t>sellerie-du-bab@orange.fr</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
-          <t>boneco-so-danca-400x400-2.jpg</t>
+          <t>cadence-cheval-mon-ami.jpg</t>
         </is>
       </c>
     </row>
@@ -1858,7 +1834,6 @@
           <t>168 bis, Rue de Charonne</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>+33 1 43 73 19 69</t>
@@ -1886,7 +1861,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>71854920_2390136477748670_1885549488290922496_n.jpg</t>
+          <t>duo-style.jpg</t>
         </is>
       </c>
     </row>
@@ -1943,7 +1918,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>348273482_280453324408988_3212622588314026301_n.jpg</t>
+          <t>fame-la-maison-de-la-danse.jpg</t>
         </is>
       </c>
     </row>
@@ -2000,7 +1975,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>boneco-so-danca-400x400-2.jpg</t>
+          <t>avant-scene.jpg</t>
         </is>
       </c>
     </row>
@@ -2025,7 +2000,6 @@
           <t>11, rue Auguste Comte</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
           <t>33 380 657 524</t>
@@ -2041,11 +2015,9 @@
           <t>https://www.instagram.com/boutiqueauxarabesques/</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
-          <t>programar-europa-1.jpg</t>
+          <t>la-boutique-aux-arabesques.jpg</t>
         </is>
       </c>
     </row>
@@ -2102,7 +2074,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>305201625_596686362058266_6288672461468767271_n.png</t>
+          <t>o-royaume-de-la-danse.png</t>
         </is>
       </c>
     </row>
@@ -2159,7 +2131,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>276055682_5056532941034427_6368756080633468488_n.jpg</t>
+          <t>dansea.jpg</t>
         </is>
       </c>
     </row>
@@ -2184,7 +2156,6 @@
           <t>46, rue de la Garenne</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>+33 6 49 55 01 68</t>
@@ -2195,7 +2166,6 @@
           <t>dansealamaud@free.fr</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
           <t>https://www.facebook.com/profile.php?id=100063792423653</t>
@@ -2208,7 +2178,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Design-sem-nome-1.jpg</t>
+          <t>danse-a-la-maud.jpg</t>
         </is>
       </c>
     </row>
@@ -2233,7 +2203,6 @@
           <t>14 Rte de la Garenne, 44700</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>+33 6 62 27 31 37</t>
@@ -2244,9 +2213,6 @@
           <t>annafranceschi@catss.fr</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr">
         <is>
           <t>catss.jpg</t>
@@ -2274,7 +2240,6 @@
           <t>395B Rue Jean Baptiste Calvignac</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>+33 4 67 16 91 26</t>
@@ -2302,7 +2267,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>245008254_4486620848120000_8770347677704494935_n.jpg</t>
+          <t>sissone.jpg</t>
         </is>
       </c>
     </row>
@@ -2327,7 +2292,6 @@
           <t>10 B, Rue du Moulin Neuf</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>06 48 84 33 94</t>
@@ -2338,8 +2302,6 @@
           <t>generationssportsetcom@orange.fr</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr">
         <is>
           <t>https://generations-sports.com/</t>
@@ -2347,7 +2309,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Design-sem-nome.jpg</t>
+          <t>generations-sports-com.jpg</t>
         </is>
       </c>
     </row>
@@ -2372,7 +2334,6 @@
           <t>89 Avenue Gabriel Peri</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>33 973 581 925</t>
@@ -2383,8 +2344,6 @@
           <t>contact@lemondedeladanse91.com</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr">
         <is>
           <t>https://www.lemondedeladanse91.com/</t>
@@ -2392,7 +2351,7 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>264238529_5009550865743159_5849123644984719875_n.jpg</t>
+          <t>le-monde-de-la-danse.jpg</t>
         </is>
       </c>
     </row>
@@ -2432,7 +2391,6 @@
           <t>mediadanse.akv@sfr.fr</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
           <t>https://www.facebook.com/p/M%C3%A9dia-Danse-100063627998416/</t>
@@ -2445,7 +2403,7 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>305049466_508905104573752_6134614782747218245_n.jpg</t>
+          <t>media-danse.jpg</t>
         </is>
       </c>
     </row>
@@ -2485,12 +2443,9 @@
           <t>boutique.letsdance@gmail.com</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr">
         <is>
-          <t>programar-europa-2.jpg</t>
+          <t>lets-dance.jpg</t>
         </is>
       </c>
     </row>
@@ -2510,8 +2465,6 @@
           <t>les-ulis</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
           <t>33 768 153 647</t>
@@ -2539,7 +2492,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>241190313_1476071486093277_1169596155638228568_n.png</t>
+          <t>claq-co.png</t>
         </is>
       </c>
     </row>
@@ -2564,7 +2517,6 @@
           <t>352 Chem. des Vergers, 06140</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
           <t>+33 6 64 04 66 85</t>
@@ -2592,7 +2544,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>15284998_224586711300495_1989407113952420855_n.jpg</t>
+          <t>la-boutique-danse.jpg</t>
         </is>
       </c>
     </row>
@@ -2632,8 +2584,6 @@
           <t>dansedescouleurs@yahoo.fr</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr">
         <is>
           <t>https://dansedescouleurs.com/355-so-danca</t>
@@ -2641,7 +2591,7 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>308518166_8014386921967647_5394266450519407410_n.jpg</t>
+          <t>danse-des-couleurs.jpg</t>
         </is>
       </c>
     </row>
@@ -2681,8 +2631,6 @@
           <t>tutu-et-cie@orange.fr</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
           <t>https://www.tutu-et-cie.com/</t>
@@ -2690,7 +2638,7 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>365779189_122096738642018167_3417460087456885942_n.jpg</t>
+          <t>tutu-cie.jpg</t>
         </is>
       </c>
     </row>
@@ -2747,7 +2695,7 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>boneco-so-danca-400x400-2.jpg</t>
+          <t>tutu-et-compagnie.jpg</t>
         </is>
       </c>
     </row>
@@ -2804,7 +2752,7 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>300396771_553363986575172_2492663777860476436_n.jpg</t>
+          <t>cadence-boutique-de-la-danse.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update smart logo mapping script and fix manual image assignments for Rey Dance and Avant-Scene
</commit_message>
<xml_diff>
--- a/sodanca-france-airtable-import.xlsx
+++ b/sodanca-france-airtable-import.xlsx
@@ -4,7 +4,7 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Cidades" sheetId="1" state="visible" r:id="rId1"/>
@@ -21,7 +21,6 @@
   <fonts count="3">
     <font>
       <name val="Calibri"/>
-      <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
@@ -31,7 +30,10 @@
       <b val="1"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Calibri"/>
+      <color theme="10"/>
+      <sz val="11"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="3">
@@ -43,7 +45,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DCE6F1"/>
+        <fgColor rgb="FFDCE6F1"/>
       </patternFill>
     </fill>
   </fills>
@@ -67,9 +69,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -142,7 +144,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -185,71 +187,13 @@
     <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:ea typeface="Arial"/>
+        <a:cs typeface="Arial"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:ea typeface="Arial"/>
+        <a:cs typeface="Arial"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -257,7 +201,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -280,7 +224,7 @@
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -371,7 +315,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -393,11 +337,9 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
+          <a:path path="circle"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -412,26 +354,23 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
+          <a:path path="circle"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:C30"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
@@ -891,29 +830,31 @@
       </c>
     </row>
   </sheetData>
+  <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" useFirstPageNumber="0" pageOrder="downThenOver" usePrinterDefaults="1" blackAndWhite="0" draft="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:K37"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="35.7109375" customWidth="1" min="1" max="1"/>
+    <col width="34.421875" customWidth="1" min="2" max="2"/>
+    <col width="24.7109375" customWidth="1" min="3" max="3"/>
+    <col width="47.00390625" customWidth="1" min="4" max="4"/>
+    <col width="60.00390625" customWidth="1" min="5" max="5"/>
+    <col width="20.421875" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="30" customWidth="1" min="8" max="8"/>
     <col width="36" customWidth="1" min="9" max="9"/>
-    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="119.57421875" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
@@ -2396,9 +2337,9 @@
           <t>https://www.facebook.com/p/M%C3%A9dia-Danse-100063627998416/</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>https://www.qualidanse.fr/?fbclid=IwY2xjawEQ3UBleHRuA2FlbQIxMAABHfBnFQeB9rpmVUR96NUfx9nSS5A8CDvph79LjFVUAvjekhceAGOGyX9XgA_aem_P87hbkw2A25ySPhXpM3IpA</t>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.qualidanse.fr/</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2757,6 +2698,11 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId1"/>
+  </hyperlinks>
+  <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" useFirstPageNumber="0" pageOrder="downThenOver" usePrinterDefaults="1" blackAndWhite="0" draft="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
 </worksheet>
 </file>
</xml_diff>